<commit_message>
Add final presentation and project reports
</commit_message>
<xml_diff>
--- a/outputs/analysis_outputs.xlsx
+++ b/outputs/analysis_outputs.xlsx
@@ -2392,13 +2392,13 @@
         <v>2006</v>
       </c>
       <c r="F7">
-        <v>40.39030179162714</v>
+        <v>40.39030179162713</v>
       </c>
       <c r="G7">
         <v>104.0870194622161</v>
       </c>
       <c r="H7">
-        <v>-63.69671767058895</v>
+        <v>-63.69671767058896</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2418,13 +2418,13 @@
         <v>2007</v>
       </c>
       <c r="F8">
-        <v>73.22677328467023</v>
+        <v>73.22677328467026</v>
       </c>
       <c r="G8">
         <v>112.4858950474131</v>
       </c>
       <c r="H8">
-        <v>-39.25912176274289</v>
+        <v>-39.25912176274286</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -2450,7 +2450,7 @@
         <v>145.0024206335535</v>
       </c>
       <c r="H9">
-        <v>-26.4272358726605</v>
+        <v>-26.42723587266048</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -2502,7 +2502,7 @@
         <v>117.5332871389736</v>
       </c>
       <c r="H11">
-        <v>41.80329694491091</v>
+        <v>41.80329694491085</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -2528,7 +2528,7 @@
         <v>159.2672075909054</v>
       </c>
       <c r="H12">
-        <v>-21.22003782677663</v>
+        <v>-21.2200378267766</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -2554,7 +2554,7 @@
         <v>156.4620533138775</v>
       </c>
       <c r="H13">
-        <v>32.85900721156659</v>
+        <v>32.85900721156662</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -2710,7 +2710,7 @@
         <v>91.46634216714887</v>
       </c>
       <c r="H19">
-        <v>24.11898627760301</v>
+        <v>24.118986277603</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -2730,13 +2730,13 @@
         <v>2019</v>
       </c>
       <c r="F20">
-        <v>82.17150359292458</v>
+        <v>82.17150359292459</v>
       </c>
       <c r="G20">
         <v>80.97845493219413</v>
       </c>
       <c r="H20">
-        <v>1.193048660730454</v>
+        <v>1.193048660730469</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -2808,13 +2808,13 @@
         <v>2022</v>
       </c>
       <c r="F23">
-        <v>91.22979234346801</v>
+        <v>91.22979234346803</v>
       </c>
       <c r="G23">
         <v>111.0495678124224</v>
       </c>
       <c r="H23">
-        <v>-19.81977546895438</v>
+        <v>-19.81977546895435</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -2938,13 +2938,13 @@
         <v>2018</v>
       </c>
       <c r="F28">
-        <v>63.15457031779584</v>
+        <v>63.1545703177959</v>
       </c>
       <c r="G28">
         <v>91.46634216714887</v>
       </c>
       <c r="H28">
-        <v>-28.31177184935302</v>
+        <v>-28.31177184935297</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -2964,13 +2964,13 @@
         <v>2019</v>
       </c>
       <c r="F29">
-        <v>181.4369545065899</v>
+        <v>181.4369545065897</v>
       </c>
       <c r="G29">
         <v>80.97845493219413</v>
       </c>
       <c r="H29">
-        <v>100.4584995743957</v>
+        <v>100.4584995743956</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -3016,13 +3016,13 @@
         <v>2021</v>
       </c>
       <c r="F31">
-        <v>67.94738141598944</v>
+        <v>67.94738141598947</v>
       </c>
       <c r="G31">
         <v>84.18803408202911</v>
       </c>
       <c r="H31">
-        <v>-16.24065266603967</v>
+        <v>-16.24065266603964</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -3042,13 +3042,13 @@
         <v>2022</v>
       </c>
       <c r="F32">
-        <v>58.99431531959123</v>
+        <v>58.99431531959122</v>
       </c>
       <c r="G32">
         <v>111.0495678124224</v>
       </c>
       <c r="H32">
-        <v>-52.05525249283115</v>
+        <v>-52.05525249283116</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -3068,13 +3068,13 @@
         <v>2023</v>
       </c>
       <c r="F33">
-        <v>98.81969765446271</v>
+        <v>98.81969765446274</v>
       </c>
       <c r="G33">
         <v>87.16646083620869</v>
       </c>
       <c r="H33">
-        <v>11.65323681825403</v>
+        <v>11.65323681825406</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -3146,13 +3146,13 @@
         <v>2026</v>
       </c>
       <c r="F36">
-        <v>80.40139769888849</v>
+        <v>80.40139769888847</v>
       </c>
       <c r="G36">
         <v>83.46550222856594</v>
       </c>
       <c r="H36">
-        <v>-3.064104529677451</v>
+        <v>-3.064104529677465</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -3172,13 +3172,13 @@
         <v>2003</v>
       </c>
       <c r="F37">
-        <v>38.2939972722918</v>
+        <v>38.29399727229183</v>
       </c>
       <c r="G37">
         <v>50.48295184397693</v>
       </c>
       <c r="H37">
-        <v>-12.18895457168512</v>
+        <v>-12.18895457168509</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -3198,13 +3198,13 @@
         <v>2004</v>
       </c>
       <c r="F38">
-        <v>60.59990299678401</v>
+        <v>60.59990299678405</v>
       </c>
       <c r="G38">
         <v>65.20709668450597</v>
       </c>
       <c r="H38">
-        <v>-4.60719368772196</v>
+        <v>-4.607193687721924</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -3224,13 +3224,13 @@
         <v>2005</v>
       </c>
       <c r="F39">
-        <v>51.52360386333255</v>
+        <v>51.52360386333257</v>
       </c>
       <c r="G39">
         <v>89.98426316188711</v>
       </c>
       <c r="H39">
-        <v>-38.46065929855456</v>
+        <v>-38.46065929855455</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -3250,13 +3250,13 @@
         <v>2006</v>
       </c>
       <c r="F40">
-        <v>36.26021458204826</v>
+        <v>36.26021458204832</v>
       </c>
       <c r="G40">
         <v>104.0870194622161</v>
       </c>
       <c r="H40">
-        <v>-67.82680488016783</v>
+        <v>-67.82680488016777</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -3276,13 +3276,13 @@
         <v>2007</v>
       </c>
       <c r="F41">
-        <v>32.62919581564719</v>
+        <v>32.62919581564722</v>
       </c>
       <c r="G41">
         <v>112.4858950474131</v>
       </c>
       <c r="H41">
-        <v>-79.85669923176593</v>
+        <v>-79.8566992317659</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -3302,13 +3302,13 @@
         <v>2008</v>
       </c>
       <c r="F42">
-        <v>31.52149583339568</v>
+        <v>31.52149583339565</v>
       </c>
       <c r="G42">
         <v>145.0024206335535</v>
       </c>
       <c r="H42">
-        <v>-113.4809248001578</v>
+        <v>-113.4809248001579</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -3328,13 +3328,13 @@
         <v>2009</v>
       </c>
       <c r="F43">
-        <v>87.17997823462571</v>
+        <v>87.17997823462572</v>
       </c>
       <c r="G43">
         <v>92.64121866765645</v>
       </c>
       <c r="H43">
-        <v>-5.461240433030738</v>
+        <v>-5.461240433030724</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -3354,13 +3354,13 @@
         <v>2010</v>
       </c>
       <c r="F44">
-        <v>115.2123464259027</v>
+        <v>115.2123464259028</v>
       </c>
       <c r="G44">
         <v>117.5332871389736</v>
       </c>
       <c r="H44">
-        <v>-2.320940713070897</v>
+        <v>-2.320940713070868</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -3386,7 +3386,7 @@
         <v>159.2672075909054</v>
       </c>
       <c r="H45">
-        <v>1.112466477109479</v>
+        <v>1.11246647710945</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -3406,13 +3406,13 @@
         <v>2012</v>
       </c>
       <c r="F46">
-        <v>180.764104600992</v>
+        <v>180.7641046009921</v>
       </c>
       <c r="G46">
         <v>156.4620533138775</v>
       </c>
       <c r="H46">
-        <v>24.30205128711455</v>
+        <v>24.30205128711461</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -3458,13 +3458,13 @@
         <v>2014</v>
       </c>
       <c r="F48">
-        <v>203.3609712982231</v>
+        <v>203.3609712982232</v>
       </c>
       <c r="G48">
         <v>134.6110022012553</v>
       </c>
       <c r="H48">
-        <v>68.74996909696782</v>
+        <v>68.74996909696787</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -3484,13 +3484,13 @@
         <v>2015</v>
       </c>
       <c r="F49">
-        <v>99.41860375351065</v>
+        <v>99.4186037535106</v>
       </c>
       <c r="G49">
         <v>71.0709351276987</v>
       </c>
       <c r="H49">
-        <v>28.34766862581195</v>
+        <v>28.34766862581189</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -3510,13 +3510,13 @@
         <v>2016</v>
       </c>
       <c r="F50">
-        <v>64.38856094321135</v>
+        <v>64.38856094321143</v>
       </c>
       <c r="G50">
         <v>58.53940291865257</v>
       </c>
       <c r="H50">
-        <v>5.849158024558776</v>
+        <v>5.849158024558861</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -3536,7 +3536,7 @@
         <v>2017</v>
       </c>
       <c r="F51">
-        <v>199.9537607415132</v>
+        <v>199.9537607415133</v>
       </c>
       <c r="G51">
         <v>71.09193192896605</v>
@@ -3562,13 +3562,13 @@
         <v>2018</v>
       </c>
       <c r="F52">
-        <v>132.3249016507653</v>
+        <v>132.3249016507654</v>
       </c>
       <c r="G52">
         <v>91.46634216714887</v>
       </c>
       <c r="H52">
-        <v>40.85855948361646</v>
+        <v>40.85855948361649</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -3588,13 +3588,13 @@
         <v>2019</v>
       </c>
       <c r="F53">
-        <v>75.74405073816008</v>
+        <v>75.74405073816013</v>
       </c>
       <c r="G53">
         <v>80.97845493219413</v>
       </c>
       <c r="H53">
-        <v>-5.234404194034042</v>
+        <v>-5.234404194033999</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -3614,13 +3614,13 @@
         <v>2020</v>
       </c>
       <c r="F54">
-        <v>66.21161229860054</v>
+        <v>66.21161229860056</v>
       </c>
       <c r="G54">
         <v>52.18596800901351</v>
       </c>
       <c r="H54">
-        <v>14.02564428958703</v>
+        <v>14.02564428958704</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -3640,13 +3640,13 @@
         <v>2021</v>
       </c>
       <c r="F55">
-        <v>10.2846964427299</v>
+        <v>10.28469644272992</v>
       </c>
       <c r="G55">
         <v>84.18803408202911</v>
       </c>
       <c r="H55">
-        <v>-73.90333763929921</v>
+        <v>-73.90333763929918</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -3666,13 +3666,13 @@
         <v>2022</v>
       </c>
       <c r="F56">
-        <v>32.365831773689</v>
+        <v>32.36583177368905</v>
       </c>
       <c r="G56">
         <v>111.0495678124224</v>
       </c>
       <c r="H56">
-        <v>-78.68373603873339</v>
+        <v>-78.68373603873334</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -3692,13 +3692,13 @@
         <v>2023</v>
       </c>
       <c r="F57">
-        <v>88.3702504129751</v>
+        <v>88.37025041297508</v>
       </c>
       <c r="G57">
         <v>87.16646083620869</v>
       </c>
       <c r="H57">
-        <v>1.203789576766411</v>
+        <v>1.203789576766397</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -3718,13 +3718,13 @@
         <v>2024</v>
       </c>
       <c r="F58">
-        <v>101.1146648093409</v>
+        <v>101.1146648093408</v>
       </c>
       <c r="G58">
         <v>82.64303534752932</v>
       </c>
       <c r="H58">
-        <v>18.47162946181155</v>
+        <v>18.47162946181152</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -3744,13 +3744,13 @@
         <v>2025</v>
       </c>
       <c r="F59">
-        <v>88.96446148460485</v>
+        <v>88.96446148460484</v>
       </c>
       <c r="G59">
         <v>69.14264822134388</v>
       </c>
       <c r="H59">
-        <v>19.82181326326098</v>
+        <v>19.82181326326096</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -3770,13 +3770,13 @@
         <v>2026</v>
       </c>
       <c r="F60">
-        <v>69.22713751966644</v>
+        <v>69.22713751966646</v>
       </c>
       <c r="G60">
         <v>83.46550222856594</v>
       </c>
       <c r="H60">
-        <v>-14.2383647088995</v>
+        <v>-14.23836470889948</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -3796,13 +3796,13 @@
         <v>2020</v>
       </c>
       <c r="F61">
-        <v>170.5151160789521</v>
+        <v>170.5151160789522</v>
       </c>
       <c r="G61">
         <v>52.18596800901351</v>
       </c>
       <c r="H61">
-        <v>118.3291480699386</v>
+        <v>118.3291480699387</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -3822,13 +3822,13 @@
         <v>2021</v>
       </c>
       <c r="F62">
-        <v>43.45318448245946</v>
+        <v>43.45318448245949</v>
       </c>
       <c r="G62">
         <v>84.18803408202911</v>
       </c>
       <c r="H62">
-        <v>-40.73484959956964</v>
+        <v>-40.73484959956961</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -3848,13 +3848,13 @@
         <v>2022</v>
       </c>
       <c r="F63">
-        <v>50.13511851239156</v>
+        <v>50.13511851239159</v>
       </c>
       <c r="G63">
         <v>111.0495678124224</v>
       </c>
       <c r="H63">
-        <v>-60.91444930003082</v>
+        <v>-60.9144493000308</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -3874,13 +3874,13 @@
         <v>2023</v>
       </c>
       <c r="F64">
-        <v>97.49038191441156</v>
+        <v>97.49038191441157</v>
       </c>
       <c r="G64">
         <v>87.16646083620869</v>
       </c>
       <c r="H64">
-        <v>10.32392107820287</v>
+        <v>10.32392107820289</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -3926,13 +3926,13 @@
         <v>2025</v>
       </c>
       <c r="F66">
-        <v>86.84810896968933</v>
+        <v>86.84810896968932</v>
       </c>
       <c r="G66">
         <v>69.14264822134388</v>
       </c>
       <c r="H66">
-        <v>17.70546074834546</v>
+        <v>17.70546074834544</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -3952,13 +3952,13 @@
         <v>2026</v>
       </c>
       <c r="F67">
-        <v>89.6296725256704</v>
+        <v>89.62967252567039</v>
       </c>
       <c r="G67">
         <v>83.46550222856594</v>
       </c>
       <c r="H67">
-        <v>6.164170297104462</v>
+        <v>6.164170297104448</v>
       </c>
     </row>
   </sheetData>
@@ -4005,13 +4005,13 @@
         <v>26</v>
       </c>
       <c r="D2">
-        <v>10.13183095505557</v>
+        <v>10.13183095505558</v>
       </c>
       <c r="E2">
         <v>35.32816650077925</v>
       </c>
       <c r="F2">
-        <v>48.95190574667282</v>
+        <v>48.95190574667281</v>
       </c>
       <c r="G2">
         <v>0.4470151332353819</v>
@@ -4028,7 +4028,7 @@
         <v>24</v>
       </c>
       <c r="D3">
-        <v>-5.407059357604319</v>
+        <v>-5.4070593576043</v>
       </c>
       <c r="E3">
         <v>35.9482123254891</v>
@@ -4051,16 +4051,16 @@
         <v>9</v>
       </c>
       <c r="D4">
-        <v>17.96027252948568</v>
+        <v>17.96027252948567</v>
       </c>
       <c r="E4">
-        <v>40.10955731568598</v>
+        <v>40.10955731568595</v>
       </c>
       <c r="F4">
-        <v>52.5105990970917</v>
+        <v>52.51059909709167</v>
       </c>
       <c r="G4">
-        <v>0.5491144320459386</v>
+        <v>0.5491144320459385</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -4074,7 +4074,7 @@
         <v>7</v>
       </c>
       <c r="D5">
-        <v>7.571707068338829</v>
+        <v>7.571707068338843</v>
       </c>
       <c r="E5">
         <v>36.6143638967961</v>
@@ -4083,7 +4083,7 @@
         <v>53.23033478323661</v>
       </c>
       <c r="G5">
-        <v>0.5391371932907426</v>
+        <v>0.5391371932907427</v>
       </c>
     </row>
   </sheetData>

</xml_diff>